<commit_message>
unificar la de dinamica forestal.
</commit_message>
<xml_diff>
--- a/Selva Viva/test.xlsx
+++ b/Selva Viva/test.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q132"/>
+  <dimension ref="A1:P132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,30 +481,25 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Type 2</t>
+          <t>sample-ID</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>sample-ID</t>
+          <t>[N]</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>[N]</t>
+          <t>[C_b]%</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>[C_b]%</t>
+          <t>δ15N (‰ v.s. V-PDB)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>δ15N (‰ v.s. V-PDB)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>bulk_δ13C (‰ v.s.V-PDB)</t>
         </is>
@@ -546,22 +541,21 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>p74-8859</t>
         </is>
       </c>
+      <c r="M2" t="n">
+        <v>0.01519611827639625</v>
+      </c>
       <c r="N2" t="n">
-        <v>0.01519611827639625</v>
+        <v>0.3990582769402648</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3990582769402648</v>
+        <v>0.5</v>
       </c>
       <c r="P2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q2" t="n">
         <v>-34.77</v>
       </c>
     </row>
@@ -601,22 +595,21 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>p74-8849</t>
         </is>
       </c>
+      <c r="M3" t="n">
+        <v>0.0157979699642389</v>
+      </c>
       <c r="N3" t="n">
-        <v>0.0157979699642389</v>
+        <v>0.4892875807439671</v>
       </c>
       <c r="O3" t="n">
-        <v>0.4892875807439671</v>
+        <v>0.44</v>
       </c>
       <c r="P3" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="Q3" t="n">
         <v>-33.24</v>
       </c>
     </row>
@@ -656,22 +649,21 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>p74-8853</t>
         </is>
       </c>
+      <c r="M4" t="n">
+        <v>0.01315526705850149</v>
+      </c>
       <c r="N4" t="n">
-        <v>0.01315526705850149</v>
+        <v>0.4473774700942126</v>
       </c>
       <c r="O4" t="n">
-        <v>0.4473774700942126</v>
+        <v>-0.42</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.42</v>
-      </c>
-      <c r="Q4" t="n">
         <v>-34.64</v>
       </c>
     </row>
@@ -711,22 +703,21 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>p74-8863</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>0.01887504041753914</v>
+      </c>
       <c r="N5" t="n">
-        <v>0.01887504041753914</v>
+        <v>0.4521728216082592</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4521728216082592</v>
+        <v>-0.82</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="Q5" t="n">
         <v>-34.43</v>
       </c>
     </row>
@@ -766,22 +757,21 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>p74-8863</t>
         </is>
       </c>
+      <c r="M6" t="n">
+        <v>0.01887504041753914</v>
+      </c>
       <c r="N6" t="n">
-        <v>0.01887504041753914</v>
+        <v>0.4521728216082592</v>
       </c>
       <c r="O6" t="n">
-        <v>0.4521728216082592</v>
+        <v>-0.82</v>
       </c>
       <c r="P6" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="Q6" t="n">
         <v>-34.43</v>
       </c>
     </row>
@@ -821,22 +811,21 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>p74-8854</t>
         </is>
       </c>
+      <c r="M7" t="n">
+        <v>0.02065846271337194</v>
+      </c>
       <c r="N7" t="n">
-        <v>0.02065846271337194</v>
+        <v>0.3932217774359631</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3932217774359631</v>
+        <v>-0.3</v>
       </c>
       <c r="P7" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="Q7" t="n">
         <v>-31.32</v>
       </c>
     </row>
@@ -881,7 +870,6 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -919,22 +907,21 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>p74-8838</t>
         </is>
       </c>
+      <c r="M9" t="n">
+        <v>0.01506027773689399</v>
+      </c>
       <c r="N9" t="n">
-        <v>0.01506027773689399</v>
+        <v>0.4810743319827603</v>
       </c>
       <c r="O9" t="n">
-        <v>0.4810743319827603</v>
+        <v>0.25</v>
       </c>
       <c r="P9" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Q9" t="n">
         <v>-33.65</v>
       </c>
     </row>
@@ -974,22 +961,21 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>p74-8840</t>
         </is>
       </c>
+      <c r="M10" t="n">
+        <v>0.013054872322637</v>
+      </c>
       <c r="N10" t="n">
-        <v>0.013054872322637</v>
+        <v>0.4551252723799056</v>
       </c>
       <c r="O10" t="n">
-        <v>0.4551252723799056</v>
+        <v>-1.16</v>
       </c>
       <c r="P10" t="n">
-        <v>-1.16</v>
-      </c>
-      <c r="Q10" t="n">
         <v>-34.88</v>
       </c>
     </row>
@@ -1029,22 +1015,21 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>p70-3622</t>
         </is>
       </c>
+      <c r="M11" t="n">
+        <v>0.01468680313508528</v>
+      </c>
       <c r="N11" t="n">
-        <v>0.01468680313508528</v>
+        <v>0.4178782536686835</v>
       </c>
       <c r="O11" t="n">
-        <v>0.4178782536686835</v>
+        <v>1.41</v>
       </c>
       <c r="P11" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="Q11" t="n">
         <v>-33.8</v>
       </c>
     </row>
@@ -1084,22 +1069,21 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>p70-3629</t>
         </is>
       </c>
+      <c r="M12" t="n">
+        <v>0.03545007406100038</v>
+      </c>
       <c r="N12" t="n">
-        <v>0.03545007406100038</v>
+        <v>0.4812524582095935</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4812524582095935</v>
+        <v>1.94</v>
       </c>
       <c r="P12" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="Q12" t="n">
         <v>-32.25</v>
       </c>
     </row>
@@ -1139,22 +1123,21 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>p70-3623</t>
         </is>
       </c>
+      <c r="M13" t="n">
+        <v>0.02344245815416083</v>
+      </c>
       <c r="N13" t="n">
-        <v>0.02344245815416083</v>
+        <v>0.4632356375118532</v>
       </c>
       <c r="O13" t="n">
-        <v>0.4632356375118532</v>
+        <v>1.86</v>
       </c>
       <c r="P13" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="Q13" t="n">
         <v>-33.18</v>
       </c>
     </row>
@@ -1194,22 +1177,21 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>p70-3654</t>
         </is>
       </c>
+      <c r="M14" t="n">
+        <v>0.02201823142746578</v>
+      </c>
       <c r="N14" t="n">
-        <v>0.02201823142746578</v>
+        <v>0.3956347601824302</v>
       </c>
       <c r="O14" t="n">
-        <v>0.3956347601824302</v>
+        <v>1.86</v>
       </c>
       <c r="P14" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="Q14" t="n">
         <v>-33.86</v>
       </c>
     </row>
@@ -1249,22 +1231,21 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>p70-3658</t>
         </is>
       </c>
+      <c r="M15" t="n">
+        <v>0.022130638</v>
+      </c>
       <c r="N15" t="n">
-        <v>0.022130638</v>
+        <v>0.436691485</v>
       </c>
       <c r="O15" t="n">
-        <v>0.436691485</v>
+        <v>2.122085858585857</v>
       </c>
       <c r="P15" t="n">
-        <v>2.122085858585857</v>
-      </c>
-      <c r="Q15" t="n">
         <v>-33.32435503711559</v>
       </c>
     </row>
@@ -1306,22 +1287,21 @@
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>p70-3658</t>
         </is>
       </c>
+      <c r="M16" t="n">
+        <v>0.022130638</v>
+      </c>
       <c r="N16" t="n">
-        <v>0.022130638</v>
+        <v>0.436691485</v>
       </c>
       <c r="O16" t="n">
-        <v>0.436691485</v>
+        <v>2.122085858585857</v>
       </c>
       <c r="P16" t="n">
-        <v>2.122085858585857</v>
-      </c>
-      <c r="Q16" t="n">
         <v>-33.32435503711559</v>
       </c>
     </row>
@@ -1361,22 +1341,21 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>p70-3634</t>
         </is>
       </c>
+      <c r="M17" t="n">
+        <v>0.01173829239074074</v>
+      </c>
       <c r="N17" t="n">
-        <v>0.01173829239074074</v>
+        <v>0.4273580210356233</v>
       </c>
       <c r="O17" t="n">
-        <v>0.4273580210356233</v>
+        <v>0.86</v>
       </c>
       <c r="P17" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="Q17" t="n">
         <v>-35.61</v>
       </c>
     </row>
@@ -1416,22 +1395,21 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>p70-3642</t>
         </is>
       </c>
+      <c r="M18" t="n">
+        <v>0.01994461056810911</v>
+      </c>
       <c r="N18" t="n">
-        <v>0.01994461056810911</v>
+        <v>0.4625106483743614</v>
       </c>
       <c r="O18" t="n">
-        <v>0.4625106483743614</v>
+        <v>1.91</v>
       </c>
       <c r="P18" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="Q18" t="n">
         <v>-31.42</v>
       </c>
     </row>
@@ -1476,7 +1454,6 @@
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1514,22 +1491,21 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>p70-3649</t>
         </is>
       </c>
+      <c r="M20" t="n">
+        <v>0.021352396</v>
+      </c>
       <c r="N20" t="n">
-        <v>0.021352396</v>
+        <v>0.483725522</v>
       </c>
       <c r="O20" t="n">
-        <v>0.483725522</v>
+        <v>2.737714646464645</v>
       </c>
       <c r="P20" t="n">
-        <v>2.737714646464645</v>
-      </c>
-      <c r="Q20" t="n">
         <v>-31.18964284199364</v>
       </c>
     </row>
@@ -1569,22 +1545,21 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>p72-8689</t>
         </is>
       </c>
+      <c r="M21" t="n">
+        <v>0.015163699</v>
+      </c>
       <c r="N21" t="n">
-        <v>0.015163699</v>
+        <v>0.468505884</v>
       </c>
       <c r="O21" t="n">
-        <v>0.468505884</v>
+        <v>2.74851515151515</v>
       </c>
       <c r="P21" t="n">
-        <v>2.74851515151515</v>
-      </c>
-      <c r="Q21" t="n">
         <v>-32.67466002120891</v>
       </c>
     </row>
@@ -1624,22 +1599,21 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>p72-8804</t>
         </is>
       </c>
+      <c r="M22" t="n">
+        <v>0.016758675</v>
+      </c>
       <c r="N22" t="n">
-        <v>0.016758675</v>
+        <v>0.473760231</v>
       </c>
       <c r="O22" t="n">
-        <v>0.473760231</v>
+        <v>1.76566919191919</v>
       </c>
       <c r="P22" t="n">
-        <v>1.76566919191919</v>
-      </c>
-      <c r="Q22" t="n">
         <v>-34.8712479321315</v>
       </c>
     </row>
@@ -1679,22 +1653,21 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>p72-8690</t>
         </is>
       </c>
+      <c r="M23" t="n">
+        <v>0.039906421</v>
+      </c>
       <c r="N23" t="n">
-        <v>0.039906421</v>
+        <v>0.432175376</v>
       </c>
       <c r="O23" t="n">
-        <v>0.432175376</v>
+        <v>2.370497474747473</v>
       </c>
       <c r="P23" t="n">
-        <v>2.370497474747473</v>
-      </c>
-      <c r="Q23" t="n">
         <v>-29.56024899257688</v>
       </c>
     </row>
@@ -1734,22 +1707,21 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>p72-8688</t>
         </is>
       </c>
+      <c r="M24" t="n">
+        <v>0.026106295</v>
+      </c>
       <c r="N24" t="n">
-        <v>0.026106295</v>
+        <v>0.456459654</v>
       </c>
       <c r="O24" t="n">
-        <v>0.456459654</v>
+        <v>2.867320707070705</v>
       </c>
       <c r="P24" t="n">
-        <v>2.867320707070705</v>
-      </c>
-      <c r="Q24" t="n">
         <v>-30.49869734888653</v>
       </c>
     </row>
@@ -1789,22 +1761,21 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>p72-8803</t>
         </is>
       </c>
+      <c r="M25" t="n">
+        <v>0.013534934</v>
+      </c>
       <c r="N25" t="n">
-        <v>0.013534934</v>
+        <v>0.4586319</v>
       </c>
       <c r="O25" t="n">
-        <v>0.4586319</v>
+        <v>2.284093434343433</v>
       </c>
       <c r="P25" t="n">
-        <v>2.284093434343433</v>
-      </c>
-      <c r="Q25" t="n">
         <v>-32.93247550371157</v>
       </c>
     </row>
@@ -1844,22 +1815,21 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>p72-8699</t>
         </is>
       </c>
+      <c r="M26" t="n">
+        <v>0.019942396</v>
+      </c>
       <c r="N26" t="n">
-        <v>0.019942396</v>
+        <v>0.460964682</v>
       </c>
       <c r="O26" t="n">
-        <v>0.460964682</v>
+        <v>1.160840909090907</v>
       </c>
       <c r="P26" t="n">
-        <v>1.160840909090907</v>
-      </c>
-      <c r="Q26" t="n">
         <v>-34.56186935312832</v>
       </c>
     </row>
@@ -1899,22 +1869,21 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>p72-8695</t>
         </is>
       </c>
+      <c r="M27" t="n">
+        <v>0.019071872</v>
+      </c>
       <c r="N27" t="n">
-        <v>0.019071872</v>
+        <v>0.460067295</v>
       </c>
       <c r="O27" t="n">
-        <v>0.460067295</v>
+        <v>2.867320707070705</v>
       </c>
       <c r="P27" t="n">
-        <v>2.867320707070705</v>
-      </c>
-      <c r="Q27" t="n">
         <v>-33.52029480381761</v>
       </c>
     </row>
@@ -1954,22 +1923,21 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>p72-8811</t>
         </is>
       </c>
+      <c r="M28" t="n">
+        <v>0.021918119</v>
+      </c>
       <c r="N28" t="n">
-        <v>0.021918119</v>
+        <v>0.409271254</v>
       </c>
       <c r="O28" t="n">
-        <v>0.409271254</v>
+        <v>1.970878787878786</v>
       </c>
       <c r="P28" t="n">
-        <v>1.970878787878786</v>
-      </c>
-      <c r="Q28" t="n">
         <v>-33.44810646871687</v>
       </c>
     </row>
@@ -2009,22 +1977,21 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>p72-8697</t>
         </is>
       </c>
+      <c r="M29" t="n">
+        <v>0.01496271</v>
+      </c>
       <c r="N29" t="n">
-        <v>0.01496271</v>
+        <v>0.480305405</v>
       </c>
       <c r="O29" t="n">
-        <v>0.480305405</v>
+        <v>1.290446969696968</v>
       </c>
       <c r="P29" t="n">
-        <v>1.290446969696968</v>
-      </c>
-      <c r="Q29" t="n">
         <v>-30.84932640509014</v>
       </c>
     </row>
@@ -2064,22 +2031,21 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>p69-3605</t>
         </is>
       </c>
+      <c r="M30" t="n">
+        <v>0.02213145516022583</v>
+      </c>
       <c r="N30" t="n">
-        <v>0.02213145516022583</v>
+        <v>0.4282614261488554</v>
       </c>
       <c r="O30" t="n">
-        <v>0.4282614261488554</v>
+        <v>0.46</v>
       </c>
       <c r="P30" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="Q30" t="n">
         <v>-31.85</v>
       </c>
     </row>
@@ -2119,22 +2085,21 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>p69-3605</t>
         </is>
       </c>
+      <c r="M31" t="n">
+        <v>0.02213145516022583</v>
+      </c>
       <c r="N31" t="n">
-        <v>0.02213145516022583</v>
+        <v>0.4282614261488554</v>
       </c>
       <c r="O31" t="n">
-        <v>0.4282614261488554</v>
+        <v>0.46</v>
       </c>
       <c r="P31" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="Q31" t="n">
         <v>-31.85</v>
       </c>
     </row>
@@ -2174,22 +2139,21 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>p69-8617</t>
         </is>
       </c>
+      <c r="M32" t="n">
+        <v>0.01853964833900083</v>
+      </c>
       <c r="N32" t="n">
-        <v>0.01853964833900083</v>
+        <v>0.4430114955907127</v>
       </c>
       <c r="O32" t="n">
-        <v>0.4430114955907127</v>
+        <v>2.34</v>
       </c>
       <c r="P32" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="Q32" t="n">
         <v>-32.61</v>
       </c>
     </row>
@@ -2229,22 +2193,21 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>p69-8898</t>
         </is>
       </c>
+      <c r="M33" t="n">
+        <v>0.02685294930046833</v>
+      </c>
       <c r="N33" t="n">
-        <v>0.02685294930046833</v>
+        <v>0.4356585352943561</v>
       </c>
       <c r="O33" t="n">
-        <v>0.4356585352943561</v>
+        <v>0.66</v>
       </c>
       <c r="P33" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="Q33" t="n">
         <v>-33.2</v>
       </c>
     </row>
@@ -2284,22 +2247,21 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>p69-3609</t>
         </is>
       </c>
+      <c r="M34" t="n">
+        <v>0.02341087029895825</v>
+      </c>
       <c r="N34" t="n">
-        <v>0.02341087029895825</v>
+        <v>0.433943697942952</v>
       </c>
       <c r="O34" t="n">
-        <v>0.433943697942952</v>
+        <v>-0.63</v>
       </c>
       <c r="P34" t="n">
-        <v>-0.63</v>
-      </c>
-      <c r="Q34" t="n">
         <v>-32.26</v>
       </c>
     </row>
@@ -2339,22 +2301,21 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>p69-3606</t>
         </is>
       </c>
+      <c r="M35" t="n">
+        <v>0.02485796670088971</v>
+      </c>
       <c r="N35" t="n">
-        <v>0.02485796670088971</v>
+        <v>0.4378430142968719</v>
       </c>
       <c r="O35" t="n">
-        <v>0.4378430142968719</v>
+        <v>0.12</v>
       </c>
       <c r="P35" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="Q35" t="n">
         <v>-31.98</v>
       </c>
     </row>
@@ -2394,22 +2355,21 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>p69-8895</t>
         </is>
       </c>
+      <c r="M36" t="n">
+        <v>0.02466862000311886</v>
+      </c>
       <c r="N36" t="n">
-        <v>0.02466862000311886</v>
+        <v>0.4874293332468896</v>
       </c>
       <c r="O36" t="n">
-        <v>0.4874293332468896</v>
+        <v>2.82</v>
       </c>
       <c r="P36" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="Q36" t="n">
         <v>-36.94</v>
       </c>
     </row>
@@ -2449,22 +2409,21 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>p69-3619</t>
         </is>
       </c>
+      <c r="M37" t="n">
+        <v>0.01915534221097701</v>
+      </c>
       <c r="N37" t="n">
-        <v>0.01915534221097701</v>
+        <v>0.4350616092673997</v>
       </c>
       <c r="O37" t="n">
-        <v>0.4350616092673997</v>
+        <v>-0.12</v>
       </c>
       <c r="P37" t="n">
-        <v>-0.12</v>
-      </c>
-      <c r="Q37" t="n">
         <v>-34.07</v>
       </c>
     </row>
@@ -2504,22 +2463,21 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>p69-3612</t>
         </is>
       </c>
+      <c r="M38" t="n">
+        <v>0.0144700480896215</v>
+      </c>
       <c r="N38" t="n">
-        <v>0.0144700480896215</v>
+        <v>0.4792818843283498</v>
       </c>
       <c r="O38" t="n">
-        <v>0.4792818843283498</v>
+        <v>-0.86</v>
       </c>
       <c r="P38" t="n">
-        <v>-0.86</v>
-      </c>
-      <c r="Q38" t="n">
         <v>-31.62</v>
       </c>
     </row>
@@ -2559,22 +2517,21 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>p69-8892</t>
         </is>
       </c>
+      <c r="M39" t="n">
+        <v>0.01810419616968846</v>
+      </c>
       <c r="N39" t="n">
-        <v>0.01810419616968846</v>
+        <v>0.4657246583502926</v>
       </c>
       <c r="O39" t="n">
-        <v>0.4657246583502926</v>
+        <v>2.56</v>
       </c>
       <c r="P39" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="Q39" t="n">
         <v>-34.8</v>
       </c>
     </row>
@@ -2614,22 +2571,21 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>p69-8891</t>
         </is>
       </c>
+      <c r="M40" t="n">
+        <v>0.02990649007833678</v>
+      </c>
       <c r="N40" t="n">
-        <v>0.02990649007833678</v>
+        <v>0.442290096180273</v>
       </c>
       <c r="O40" t="n">
-        <v>0.442290096180273</v>
+        <v>-0.03</v>
       </c>
       <c r="P40" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="Q40" t="n">
         <v>-35.22</v>
       </c>
     </row>
@@ -2669,22 +2625,21 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>p68-8889</t>
         </is>
       </c>
+      <c r="M41" t="n">
+        <v>0.024841004</v>
+      </c>
       <c r="N41" t="n">
-        <v>0.024841004</v>
+        <v>0.404913041</v>
       </c>
       <c r="O41" t="n">
-        <v>0.404913041</v>
+        <v>1.312047979797978</v>
       </c>
       <c r="P41" t="n">
-        <v>1.312047979797978</v>
-      </c>
-      <c r="Q41" t="n">
         <v>-31.78777476139979</v>
       </c>
     </row>
@@ -2724,22 +2679,21 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>p68-8883</t>
         </is>
       </c>
+      <c r="M42" t="n">
+        <v>0.014952077</v>
+      </c>
       <c r="N42" t="n">
-        <v>0.014952077</v>
+        <v>0.406260288</v>
       </c>
       <c r="O42" t="n">
-        <v>0.406260288</v>
+        <v>2.392098484848483</v>
       </c>
       <c r="P42" t="n">
-        <v>2.392098484848483</v>
-      </c>
-      <c r="Q42" t="n">
         <v>-31.90121357370095</v>
       </c>
     </row>
@@ -2779,22 +2733,21 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>p68-8870</t>
         </is>
       </c>
+      <c r="M43" t="n">
+        <v>0.021749615</v>
+      </c>
       <c r="N43" t="n">
-        <v>0.021749615</v>
+        <v>0.495438619</v>
       </c>
       <c r="O43" t="n">
-        <v>0.495438619</v>
+        <v>-0.5456388888888914</v>
       </c>
       <c r="P43" t="n">
-        <v>-0.5456388888888914</v>
-      </c>
-      <c r="Q43" t="n">
         <v>-34.0256131495228</v>
       </c>
     </row>
@@ -2834,22 +2787,21 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>p68-8876</t>
         </is>
       </c>
+      <c r="M44" t="n">
+        <v>0.017456195</v>
+      </c>
       <c r="N44" t="n">
-        <v>0.017456195</v>
+        <v>0.481396993</v>
       </c>
       <c r="O44" t="n">
-        <v>0.481396993</v>
+        <v>-0.6320429292929319</v>
       </c>
       <c r="P44" t="n">
-        <v>-0.6320429292929319</v>
-      </c>
-      <c r="Q44" t="n">
         <v>-34.2009276776246</v>
       </c>
     </row>
@@ -2889,22 +2841,21 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>p68-8867</t>
         </is>
       </c>
+      <c r="M45" t="n">
+        <v>0.020640948</v>
+      </c>
       <c r="N45" t="n">
-        <v>0.020640948</v>
+        <v>0.440605127</v>
       </c>
       <c r="O45" t="n">
-        <v>0.440605127</v>
+        <v>1.538858585858584</v>
       </c>
       <c r="P45" t="n">
-        <v>1.538858585858584</v>
-      </c>
-      <c r="Q45" t="n">
         <v>-34.17514612937434</v>
       </c>
     </row>
@@ -2944,22 +2895,21 @@
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>p68-8867</t>
         </is>
       </c>
+      <c r="M46" t="n">
+        <v>0.020640948</v>
+      </c>
       <c r="N46" t="n">
-        <v>0.020640948</v>
+        <v>0.440605127</v>
       </c>
       <c r="O46" t="n">
-        <v>0.440605127</v>
+        <v>1.538858585858584</v>
       </c>
       <c r="P46" t="n">
-        <v>1.538858585858584</v>
-      </c>
-      <c r="Q46" t="n">
         <v>-34.17514612937434</v>
       </c>
     </row>
@@ -2999,22 +2949,21 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>p68-8888</t>
         </is>
       </c>
+      <c r="M47" t="n">
+        <v>0.011420399</v>
+      </c>
       <c r="N47" t="n">
-        <v>0.011420399</v>
+        <v>0.430948024</v>
       </c>
       <c r="O47" t="n">
-        <v>0.430948024</v>
+        <v>2.435300505050503</v>
       </c>
       <c r="P47" t="n">
-        <v>2.435300505050503</v>
-      </c>
-      <c r="Q47" t="n">
         <v>-34.86093531283139</v>
       </c>
     </row>
@@ -3059,7 +3008,6 @@
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -3108,7 +3056,6 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -3157,7 +3104,6 @@
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -3206,7 +3152,6 @@
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -3255,7 +3200,6 @@
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -3304,7 +3248,6 @@
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -3353,7 +3296,6 @@
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -3402,7 +3344,6 @@
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -3451,7 +3392,6 @@
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -3496,7 +3436,6 @@
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -3545,7 +3484,6 @@
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -3594,7 +3532,6 @@
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -3643,7 +3580,6 @@
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -3692,7 +3628,6 @@
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -3741,7 +3676,6 @@
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -3790,7 +3724,6 @@
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -3839,7 +3772,6 @@
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -3888,7 +3820,6 @@
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -3937,7 +3868,6 @@
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -3986,7 +3916,6 @@
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -4035,7 +3964,6 @@
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -4084,7 +4012,6 @@
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -4133,7 +4060,6 @@
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -4182,7 +4108,6 @@
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -4231,7 +4156,6 @@
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -4280,7 +4204,6 @@
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -4329,7 +4252,6 @@
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -4378,7 +4300,6 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
-      <c r="Q75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -4427,7 +4348,6 @@
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -4476,7 +4396,6 @@
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr"/>
-      <c r="Q77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -4525,7 +4444,6 @@
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -4574,7 +4492,6 @@
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr"/>
-      <c r="Q79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -4623,7 +4540,6 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -4672,7 +4588,6 @@
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -4721,7 +4636,6 @@
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -4770,7 +4684,6 @@
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -4819,7 +4732,6 @@
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -4868,7 +4780,6 @@
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -4917,7 +4828,6 @@
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr"/>
-      <c r="Q86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -4966,7 +4876,6 @@
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -5015,7 +4924,6 @@
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -5064,7 +4972,6 @@
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -5113,7 +5020,6 @@
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -5162,7 +5068,6 @@
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -5211,7 +5116,6 @@
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -5260,7 +5164,6 @@
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
-      <c r="Q93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -5309,7 +5212,6 @@
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
-      <c r="Q94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -5358,7 +5260,6 @@
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr"/>
-      <c r="Q95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -5407,7 +5308,6 @@
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr"/>
-      <c r="Q96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -5456,7 +5356,6 @@
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr"/>
-      <c r="Q97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -5505,7 +5404,6 @@
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr"/>
-      <c r="Q98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -5554,7 +5452,6 @@
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr"/>
-      <c r="Q99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -5603,7 +5500,6 @@
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
-      <c r="Q100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -5652,7 +5548,6 @@
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr"/>
-      <c r="Q101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -5701,7 +5596,6 @@
       <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr"/>
-      <c r="Q102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -5750,7 +5644,6 @@
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr"/>
-      <c r="Q103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -5799,7 +5692,6 @@
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr"/>
-      <c r="Q104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -5848,7 +5740,6 @@
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr"/>
-      <c r="Q105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -5897,7 +5788,6 @@
       <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr"/>
-      <c r="Q106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -5946,7 +5836,6 @@
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr"/>
-      <c r="Q107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -5991,7 +5880,6 @@
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr"/>
-      <c r="Q108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -6036,7 +5924,6 @@
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr"/>
-      <c r="Q109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -6081,7 +5968,6 @@
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr"/>
-      <c r="Q110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -6126,7 +6012,6 @@
       <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr"/>
-      <c r="Q111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -6171,7 +6056,6 @@
       <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr"/>
-      <c r="Q112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -6216,7 +6100,6 @@
       <c r="N113" t="inlineStr"/>
       <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr"/>
-      <c r="Q113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -6261,7 +6144,6 @@
       <c r="N114" t="inlineStr"/>
       <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr"/>
-      <c r="Q114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -6306,7 +6188,6 @@
       <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr"/>
       <c r="P115" t="inlineStr"/>
-      <c r="Q115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -6351,7 +6232,6 @@
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr"/>
-      <c r="Q116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -6396,7 +6276,6 @@
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr"/>
       <c r="P117" t="inlineStr"/>
-      <c r="Q117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -6441,7 +6320,6 @@
       <c r="N118" t="inlineStr"/>
       <c r="O118" t="inlineStr"/>
       <c r="P118" t="inlineStr"/>
-      <c r="Q118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -6486,7 +6364,6 @@
       <c r="N119" t="inlineStr"/>
       <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr"/>
-      <c r="Q119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -6531,7 +6408,6 @@
       <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr"/>
-      <c r="Q120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -6576,7 +6452,6 @@
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -6614,22 +6489,21 @@
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr"/>
       <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr">
+      <c r="L122" t="inlineStr">
         <is>
           <t>p70-3635</t>
         </is>
       </c>
+      <c r="M122" t="n">
+        <v>0.02329030068816614</v>
+      </c>
       <c r="N122" t="n">
-        <v>0.02329030068816614</v>
+        <v>0.4286406242211068</v>
       </c>
       <c r="O122" t="n">
-        <v>0.4286406242211068</v>
+        <v>0.67</v>
       </c>
       <c r="P122" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="Q122" t="n">
         <v>-34.74</v>
       </c>
     </row>
@@ -6673,16 +6547,11 @@
         </is>
       </c>
       <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr"/>
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr"/>
-      <c r="Q123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -6728,16 +6597,11 @@
           <t>2223</t>
         </is>
       </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="inlineStr"/>
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr"/>
-      <c r="Q124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -6783,16 +6647,11 @@
           <t>2230</t>
         </is>
       </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="inlineStr"/>
       <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -6838,16 +6697,11 @@
           <t>2246</t>
         </is>
       </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -6893,16 +6747,11 @@
           <t>2380</t>
         </is>
       </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr"/>
-      <c r="Q127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -6948,16 +6797,11 @@
           <t>2239</t>
         </is>
       </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr"/>
-      <c r="Q128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -7003,16 +6847,11 @@
           <t>2303</t>
         </is>
       </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr"/>
-      <c r="Q129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -7058,16 +6897,11 @@
           <t>2245</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>jh</t>
-        </is>
-      </c>
+      <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="inlineStr"/>
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr"/>
-      <c r="Q130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -7083,7 +6917,9 @@
       <c r="E131" t="n">
         <v>2025</v>
       </c>
-      <c r="F131" t="inlineStr"/>
+      <c r="F131" t="n">
+        <v>68</v>
+      </c>
       <c r="G131" t="n">
         <v>8878</v>
       </c>
@@ -7091,22 +6927,21 @@
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
-      <c r="M131" t="inlineStr">
+      <c r="L131" t="inlineStr">
         <is>
           <t>p68-8878</t>
         </is>
       </c>
+      <c r="M131" t="n">
+        <v>0.017277264</v>
+      </c>
       <c r="N131" t="n">
-        <v>0.017277264</v>
+        <v>0.437306213</v>
       </c>
       <c r="O131" t="n">
-        <v>0.437306213</v>
+        <v>1.571260101010099</v>
       </c>
       <c r="P131" t="n">
-        <v>1.571260101010099</v>
-      </c>
-      <c r="Q131" t="n">
         <v>-34.25249077412514</v>
       </c>
     </row>
@@ -7124,7 +6959,9 @@
       <c r="E132" t="n">
         <v>2025</v>
       </c>
-      <c r="F132" t="inlineStr"/>
+      <c r="F132" t="n">
+        <v>68</v>
+      </c>
       <c r="G132" t="n">
         <v>8885</v>
       </c>
@@ -7132,22 +6969,21 @@
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" t="inlineStr">
+      <c r="L132" t="inlineStr">
         <is>
           <t>p68-8885</t>
         </is>
       </c>
+      <c r="M132" t="n">
+        <v>0.015294916</v>
+      </c>
       <c r="N132" t="n">
-        <v>0.015294916</v>
+        <v>0.488282508</v>
       </c>
       <c r="O132" t="n">
-        <v>0.488282508</v>
+        <v>0.8692272727272705</v>
       </c>
       <c r="P132" t="n">
-        <v>0.8692272727272705</v>
-      </c>
-      <c r="Q132" t="n">
         <v>-33.91217433722163</v>
       </c>
     </row>

</xml_diff>